<commit_message>
Actualizar catálogo a 24 soluciones incorporando Solagro y script de monitoreo
</commit_message>
<xml_diff>
--- a/soluciones_inia_converge.xlsx
+++ b/soluciones_inia_converge.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Soluciones INIA Converge" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Soluciones INIA Converge'!$A$1:$L$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Soluciones INIA Converge'!$A$1:$L$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1857,8 +1857,64 @@
         <v/>
       </c>
     </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Vegetal Extensivo</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Agricultura De Precisión</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Solagro</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Octubre 2025 (INIA La Estanzuela)</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="G25" s="9">
+        <f>HYPERLINK("https://inia.uy/Converge/vegetal-extensivo/agricultura-de-precisión/Solagro", "Ver Ficha")</f>
+        <v/>
+      </c>
+      <c r="H25" s="9">
+        <f>HYPERLINK("https://inia.uy/sites/default/files/gras/contenidogras/Reportes/Converge/PaginasProductos/Solagro/Reporte_Solagro.pdf", "Reporte (PDF)")</f>
+        <v/>
+      </c>
+      <c r="I25" s="9">
+        <f>HYPERLINK("https://inia.uy/sites/default/files/gras/contenidogras/Reportes/Converge/PaginasProductos/Solagro/Informe_Solagro.pdf", "Extendido (PDF)")</f>
+        <v/>
+      </c>
+      <c r="J25" s="9">
+        <f>HYPERLINK("https://inia.uy/sites/default/files/gras/contenidogras/Reportes/Converge/PaginasProductos/Solagro/Testimonios_Solagro.pdf", "Testimonio (PDF)")</f>
+        <v/>
+      </c>
+      <c r="K25" s="9">
+        <f>HYPERLINK("https://inia.uy/sites/default/files/gras/contenidogras/Reportes/Converge/PaginasProductos/Solagro/Ficha_Solagro_Selenium.jpg", "Ficha Gráfica")</f>
+        <v/>
+      </c>
+      <c r="L25" s="9">
+        <f>HYPERLINK("https://solagro.com.uy/", "Web Oficial")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L24"/>
+  <autoFilter ref="A1:L25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corregir URL y metadatos de DeepAgro Soja y actualizar monitor para sellos reubicados
</commit_message>
<xml_diff>
--- a/soluciones_inia_converge.xlsx
+++ b/soluciones_inia_converge.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Soluciones INIA Converge" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soluciones INIA Converge" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Soluciones INIA Converge'!$A$1:$L$27</definedName>
@@ -1921,22 +1921,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Agricultura De Precisión</t>
+          <t>Control De Aplicaciones</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>deepagro-soja</t>
+          <t>DeepAgro Soja</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Septiembre 2023</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Noviembre 2025 a Febrero 2026 (INIA La Estanzuela - Aplicación selectiva en soja)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="G26" s="5">
-        <f>HYPERLINK("https://inia.uy/Converge/vegetal-extensivo/agricultura-de-precisión/deepagro-soja", "Ver Ficha")</f>
+        <f>HYPERLINK("https://inia.uy/Converge/vegetal-extensivo/control-de-aplicaciones/deepagro-soja", "Ver Ficha")</f>
         <v/>
       </c>
       <c r="H26" s="5">
@@ -1953,7 +1953,7 @@
         <v/>
       </c>
       <c r="I26" s="5">
-        <f>HYPERLINK("-", "Extendido (PDF)")</f>
+        <f>HYPERLINK("https://inia.uy/sites/default/files/gras/contenidogras/Reportes/Converge/PaginasProductos/DeepAgro_Soja/Informe_SprAI_Soja.pdf", "Extendido (PDF)")</f>
         <v/>
       </c>
       <c r="J26" s="5">
@@ -1965,7 +1965,7 @@
         <v/>
       </c>
       <c r="L26" s="5">
-        <f>HYPERLINK("-", "Web Oficial")</f>
+        <f>HYPERLINK("https://www.deepagro.com/", "Web Oficial")</f>
         <v/>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>(establecimiento Il Tramonto)</t>
+          <t>Instancia de verificación técnica en feedlot (Establecimiento Il Tramonto)</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">

</xml_diff>